<commit_message>
Add employee and rep data collection system (Arabic web app)
Flask + SQLite app driven by a single field schema (app/fields.py):
- employee portal via personal link with last-4-ID check, draft/submit,
  vehicle/odometer photo upload (resized, EXIF stripped)
- HR dashboard: progress, filters, review/approve/return, expiry alerts,
  WhatsApp reminder links, audit log, masked sensitive values
- Excel import (dry-run first) and export in the template layout
- login lockout, CSRF, security headers, backup script
- 35 tests; Docker/Caddy deployment files (untested), Arabic README

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0195cKRAPvS9apkqqLz2bAG2
</commit_message>
<xml_diff>
--- a/employee-data-template.xlsx
+++ b/employee-data-template.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تعليمات" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الموظفون" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المناديب" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="قاموس الحقول" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="القوائم" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="تعليمات" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="الموظفون" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="المناديب" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="قاموس الحقول" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="القوائم" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>